<commit_message>
playbook A.5 + case cross-ref: video-not-photo pair
- analysis_playbook.md: Phụ lục A.5 bang ba-dao-ham (Video vs Photo)
  Bang doi chung CASE_HEI (DUONG) vs CASE_BANANAS31 (AM)
  Quy trinh 4 buoc khi pos_r > 4: sign-corr → dist_wall → gLSR → TRACKING
  Cross-ref table: ARM row +L-46/47, DATA row +L-48
- CASE_BANANAS31.xlsx: CASE verdict=NO_SETUP-TRACKING-passive (L-47 expiry)
  TRIGGERS: T1/T2/T3 WAIT, INV=BLOCK (gLSR=1.20), archetype=MM-BAIT-B-shape
  OUTCOME: giao khoa L-46/47/48, dong ho cum #4 Aug-Oct/26
- CASE_HEI.xlsx EVENTS: cross-ref doi chung DUONG cap L-46
- docs/INDEX.md: fix broken HEI+BANANAS31 row, L-01→L-48, version 09/08
- scripts/_task_regen_lessons.py: reusable regen utility (scripts/, not archive)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANANAS31.xlsx
+++ b/docs/case_files/CASE_BANANAS31.xlsx
@@ -575,6 +575,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -607,7 +608,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>COLD_START — PENDING</t>
+          <t>NO_SETUP — TRACKING-passive. Build 06/26 het han (L-47). Ho MM-BAIT-B-shape serial, dong ho cum #4 Aug-Oct/26 [n=3 INFERENCE]. Operator signed 09/08.</t>
         </is>
       </c>
     </row>
@@ -761,7 +762,11 @@
           <t>Archetype</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>MM-BAIT-B-shape serial (INFERENCE, n=3)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -73732,9 +73737,145 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Threshold</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Ghi chu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>gLSR drop + pos rebuild</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>gLSR &lt;= 0.7 + pos_r tang 3d</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>WAIT</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Fuel nap tu reset crowd</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Volume bung ben vung gia</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>vol &gt;= 3x med14 ben &gt;= 2d</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>WAIT</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Confirm build momentum</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>GOM-A fire + yaml screen pass</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>GOM-A=TRUE + screen pass</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>WAIT</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Xem screen_thresholds.yaml</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>INV</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>gLSR &gt;= 1.2 hien tai (block entry)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>gLSR &gt;= 1.2</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>BLOCK</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Crowd da long het — mat fuel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -73745,9 +73886,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>verdict_operator</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>NO_SETUP — TRACKING-passive</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ngay_verdict</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>archetype</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>MM-BAIT-B-shape serial (INFERENCE n=3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ghi_chu</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Case giao khoa L-46/47/48 — giu lam doi chung, khong dong file</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>clock_cum_4</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Du kien Aug-Oct 2026 — theo doi gLSR drop ve &lt;= 0.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>operator_signed</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>09/08/2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>